<commit_message>
feat: expand Excel automation test suite to 36 test cases with full CRUD and multi-attendee checkin flows
</commit_message>
<xml_diff>
--- a/tests/test_cases.xlsx
+++ b/tests/test_cases.xlsx
@@ -435,15 +435,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
@@ -599,31 +599,35 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>List Active Events</t>
+          <t>Create New Event</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>/api/events?status=ACTIVE,PUBLISHED</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr"/>
+          <t>/api/events</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>{"name": "Tech Gala Expo ${timestamp}", "description": "Annual Technology Innovation Summit", "venue": "Grand Hall 1", "startDate": "2026-12-01T09:00:00.000Z", "endDate": "2026-12-01T18:00:00.000Z", "status": "ACTIVE"}</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>data.id</t>
         </is>
       </c>
     </row>
@@ -640,12 +644,12 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Get Event Details by ID</t>
+          <t>Update Event Status to Active/Public</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PUT</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -653,10 +657,14 @@
           <t>/api/events/${eventId}</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>{"status": "ACTIVE"}</t>
+        </is>
+      </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -664,7 +672,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>data.name</t>
+          <t>data.id</t>
         </is>
       </c>
     </row>
@@ -676,12 +684,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>CheckinPoints</t>
+          <t>Events</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Get Entrance Points List</t>
+          <t>Get Event Detail</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -691,7 +699,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>/api/checkin/points?eventId=${eventId}</t>
+          <t>/api/events/${eventId}</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr"/>
@@ -705,7 +713,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>data.name</t>
         </is>
       </c>
     </row>
@@ -722,35 +730,31 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Create New Entrance Gate</t>
+          <t>Get Entrance Points List</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>/api/checkin/points</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>{"eventId": "${eventId}", "name": "Excel Gate Door 1", "location": "Hall 1", "isActive": true, "sortOrder": 10}</t>
-        </is>
-      </c>
+          <t>/api/checkin/points?eventId=${eventId}</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>data.id</t>
+          <t>data</t>
         </is>
       </c>
     </row>
@@ -762,12 +766,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>CheckinPoints</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Register New Attendee</t>
+          <t>Create New Entrance Gate</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -777,17 +781,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>/api/registrations</t>
+          <t>/api/checkin/points</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>{"eventId": "${eventId}", "fullName": "Excel Tester Guest", "email": "excel.test.${timestamp}@example.com", "phone": "0899999999", "company": "Excel QA Corp"}</t>
+          <t>{"eventId": "${eventId}", "name": "VIP Entrance Gate 1", "location": "Hall A North", "isActive": true, "sortOrder": 1}</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
@@ -807,12 +811,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Checkin</t>
+          <t>Registration</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Perform Gate Check-in</t>
+          <t>Register New Attendee (Guest 1)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -822,12 +826,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>/api/checkin</t>
+          <t>/api/registrations</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>{"registrationId": "${registrationId}", "checkinPointId": "${pointId}", "method": "MANUAL"}</t>
+          <t>{"eventId": "${eventId}", "fullName": "Somchai Jaidee (Guest 1)", "email": "somchai.${timestamp}@example.com", "phone": "0811111111", "company": "Tech Corp"}</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -840,7 +844,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>data.checkin.id</t>
+          <t>data.id</t>
         </is>
       </c>
     </row>
@@ -852,36 +856,40 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>LuckyDraw</t>
+          <t>Checkin</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Fetch Prizes &amp; Eligible Count</t>
+          <t>Perform Gate Check-in (Guest 1)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>/api/prizes?eventId=${eventId}</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr"/>
+          <t>/api/checkin</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>{"registrationId": "${registrationId}", "checkinPointId": "${pointId}", "method": "MANUAL"}</t>
+        </is>
+      </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>data.checkin.id</t>
         </is>
       </c>
     </row>
@@ -893,12 +901,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>LuckyDraw</t>
+          <t>Registration</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Start Draw Session</t>
+          <t>Register New Attendee (Guest 2)</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -908,17 +916,17 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>/api/draws/start</t>
+          <t>/api/registrations</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>{"eventId": "${eventId}", "prizeId": "${prizeId}", "drawCount": 1}</t>
+          <t>{"eventId": "${eventId}", "fullName": "Siriporn Boonmee (Guest 2)", "email": "siriporn.${timestamp}@example.com", "phone": "0822222222", "company": "Innovate Ltd"}</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
@@ -938,12 +946,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>LuckyDraw</t>
+          <t>Checkin</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Execute Spin Fisher-Yates Draw</t>
+          <t>Perform Gate Check-in (Guest 2)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -953,12 +961,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>/api/draws/${drawSessionId}/spin</t>
+          <t>/api/checkin</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>{"count": 1}</t>
+          <t>{"registrationId": "${registrationId}", "checkinPointId": "${pointId}", "method": "MANUAL"}</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -967,11 +975,11 @@
         </is>
       </c>
       <c r="H12" s="2" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>data.winners</t>
+          <t>data.checkin.id</t>
         </is>
       </c>
     </row>
@@ -983,40 +991,40 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>WinnerMgmt</t>
+          <t>Registration</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Update Winner Status to ACCEPTED</t>
+          <t>Register New Attendee (Guest 3)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>PUT</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>/api/draws/winners/${winnerId}</t>
+          <t>/api/registrations</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>{"status": "ACCEPTED"}</t>
+          <t>{"eventId": "${eventId}", "fullName": "Wichai Chaichana (Guest 3)", "email": "wichai.${timestamp}@example.com", "phone": "0833333333", "company": "Digital Group"}</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>data.status</t>
+          <t>data.id</t>
         </is>
       </c>
     </row>
@@ -1028,34 +1036,1065 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
+          <t>Checkin</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Perform Gate Check-in (Guest 3)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>/api/checkin</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>{"registrationId": "${registrationId}", "checkinPointId": "${pointId}", "method": "MANUAL"}</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>data.checkin.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>TC-014</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Registration</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Register New Attendee (Guest 4)</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>/api/registrations</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>{"eventId": "${eventId}", "fullName": "Anan Srisuk (Guest 4)", "email": "anan.${timestamp}@example.com", "phone": "0844444444", "company": "Software Inc"}</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>data.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>TC-015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Checkin</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Perform Gate Check-in (Guest 4)</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>/api/checkin</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>{"registrationId": "${registrationId}", "checkinPointId": "${pointId}", "method": "MANUAL"}</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>data.checkin.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>TC-016</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Registration</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Register New Attendee (Guest 5)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>/api/registrations</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>{"eventId": "${eventId}", "fullName": "Kanya Wattana (Guest 5)", "email": "kanya.${timestamp}@example.com", "phone": "0855555555", "company": "Cloud Systems"}</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>data.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>TC-017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Registration</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Register New Attendee (Guest 6)</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>/api/registrations</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>{"eventId": "${eventId}", "fullName": "Nattapong Somboon (Guest 6)", "email": "nattapong.${timestamp}@example.com", "phone": "0866666666", "company": "Cyber Security"}</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>data.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>TC-018</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Registration</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Register New Attendee (Guest 7)</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>/api/registrations</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>{"eventId": "${eventId}", "fullName": "Piyada Rattanaporn (Guest 7)", "email": "piyada.${timestamp}@example.com", "phone": "0877777777", "company": "Data Analytics"}</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>data.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>TC-019</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Registration</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Register New Attendee (Guest 8)</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>/api/registrations</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>{"eventId": "${eventId}", "fullName": "Thanakorn Prasert (Guest 8)", "email": "thanakorn.${timestamp}@example.com", "phone": "0888888888", "company": "AI Labs"}</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>data.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>TC-020</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Registration</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Register New Attendee (Guest 9)</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>/api/registrations</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>{"eventId": "${eventId}", "fullName": "Chutima Wongwian (Guest 9)", "email": "chutima.${timestamp}@example.com", "phone": "0899999991", "company": "Media Network"}</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>data.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>TC-021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Registration</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Register New Attendee (Guest 10)</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>/api/registrations</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>{"eventId": "${eventId}", "fullName": "Phopkrit Panich (Guest 10)", "email": "phopkrit.${timestamp}@example.com", "phone": "0899999992", "company": "Finance Hub"}</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>data.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>TC-022</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Registration</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Register New Attendee (Guest 11)</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>/api/registrations</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>{"eventId": "${eventId}", "fullName": "Suthep Ruangrit (Guest 11)", "email": "suthep.${timestamp}@example.com", "phone": "0899999993", "company": "Logistics Pro"}</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>data.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>TC-023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Registration</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Register New Attendee (Guest 12)</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>/api/registrations</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>{"eventId": "${eventId}", "fullName": "Rungtiwa Kaewmanee (Guest 12)", "email": "rungtiwa.${timestamp}@example.com", "phone": "0899999994", "company": "Creative Studio"}</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>data.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>TC-024</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Registration</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Register New Attendee (Guest 13)</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>/api/registrations</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>{"eventId": "${eventId}", "fullName": "Banthit Charoen (Guest 13)", "email": "banthit.${timestamp}@example.com", "phone": "0899999995", "company": "Mobile Apps"}</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>data.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>TC-025</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Registration</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Register New Attendee (Guest 14)</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>/api/registrations</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>{"eventId": "${eventId}", "fullName": "Wanida Saetang (Guest 14)", "email": "wanida.${timestamp}@example.com", "phone": "0899999996", "company": "E-Commerce Group"}</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>data.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>TC-026</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Registration</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Register New Attendee (Guest 15)</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>/api/registrations</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>{"eventId": "${eventId}", "fullName": "Kraisorn Decha (Guest 15)", "email": "kraisorn.${timestamp}@example.com", "phone": "0899999997", "company": "Robotics Corp"}</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>data.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>TC-027</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Registration</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Register New Attendee (Guest 16)</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>/api/registrations</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>{"eventId": "${eventId}", "fullName": "Worawat Songsak (Guest 16)", "email": "worawat.${timestamp}@example.com", "phone": "0899999998", "company": "Gaming World"}</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>data.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>TC-028</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Registration</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Register New Attendee (Guest 17)</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>/api/registrations</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>{"eventId": "${eventId}", "fullName": "Jintana Phusit (Guest 17)", "email": "jintana.${timestamp}@example.com", "phone": "0812345601", "company": "Health Tech"}</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>data.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>TC-029</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Registration</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Register New Attendee (Guest 18)</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>/api/registrations</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>{"eventId": "${eventId}", "fullName": "Prasit Manop (Guest 18)", "email": "prasit.${timestamp}@example.com", "phone": "0812345602", "company": "Green Energy"}</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>data.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>TC-030</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Registration</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Register New Attendee (Guest 19)</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>/api/registrations</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>{"eventId": "${eventId}", "fullName": "Rattana Chokdee (Guest 19)", "email": "rattana.${timestamp}@example.com", "phone": "0812345603", "company": "Smart City"}</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>data.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>TC-031</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Prizes</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Create Prize for Event</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>/api/prizes</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>{"eventId": "${eventId}", "name": "Grand Prize iPhone 16 Pro", "description": "Top Lucky Draw Prize", "quantity": 5, "sortOrder": 1}</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>data.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>TC-032</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>LuckyDraw</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Fetch Prizes &amp; Eligible Count</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>/api/prizes?eventId=${eventId}</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>TC-033</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>LuckyDraw</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Start Lucky Draw Session</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>/api/draws/start</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>{"eventId": "${eventId}", "prizeId": "${prizeId}", "drawCount": 1}</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>data.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>TC-034</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>LuckyDraw</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Execute Fisher-Yates Spin Draw (1 Winner)</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>/api/draws/${drawSessionId}/spin</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>{"count": 1}</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>data.winners</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>TC-035</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
           <t>WinnerMgmt</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Update Winner Status to ACCEPTED</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>/api/draws/winners/${winnerId}</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>{"status": "ACCEPTED"}</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>data.status</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>TC-036</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>WinnerMgmt</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>Delete Winner &amp; Recalculate Quota</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>/api/draws/winners/${winnerId}</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="H14" s="2" t="n">
+      <c r="H37" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="I37" s="2" t="inlineStr">
         <is>
           <t>message</t>
         </is>

</xml_diff>